<commit_message>
actualizacion de detalles arreglado
</commit_message>
<xml_diff>
--- a/src/modules/planillas_aportes/templates/plantilla.xlsx
+++ b/src/modules/planillas_aportes/templates/plantilla.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CBES\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CBES\Documents\SISTEMAS\COTIZACIONES\BACKEND-COTIZACIONES\cotizaciones-backend-desarrollo\src\modules\planillas_aportes\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73AC7530-C0DC-4B50-8A16-F81C1543604F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6D28696-BE53-4A52-A3CF-1544E0705126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29400" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLANILLA SALARIAL" sheetId="1" r:id="rId1"/>
@@ -620,10 +620,17 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -683,13 +690,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor rgb="FF005E00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -727,52 +734,59 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 5 2" xfId="1" xr:uid="{B99F7E89-A1B7-43AF-A881-C7B51ABB3549}"/>
+    <cellStyle name="Normal 5 2 2" xfId="3" xr:uid="{9B251163-567E-4153-B316-A1D09BC4EF61}"/>
     <cellStyle name="Título 3" xfId="2" builtinId="18"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1182,34 +1196,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" ht="42" customHeight="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -1224,10 +1238,10 @@
       <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="12" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="3" t="s">
@@ -1248,7 +1262,7 @@
       <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="12" t="s">
         <v>22</v>
       </c>
       <c r="X1" s="3" t="s">
@@ -1257,28 +1271,28 @@
       <c r="Y1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="Z1" s="12" t="s">
         <v>25</v>
       </c>
       <c r="AA1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AB1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AC1" s="12" t="s">
         <v>28</v>
       </c>
       <c r="AD1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AE1" s="12" t="s">
         <v>30</v>
       </c>
       <c r="AF1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AG1" s="12" t="s">
         <v>32</v>
       </c>
       <c r="AH1" s="3" t="s">
@@ -1305,7 +1319,7 @@
       <c r="AO1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AP1" s="12" t="s">
         <v>41</v>
       </c>
       <c r="AQ1" s="3" t="s">
@@ -1320,15 +1334,58 @@
       <c r="AT1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="3" t="s">
+      <c r="AU1" s="12" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:47">
-      <c r="E2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="AT2" s="2"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
+      <c r="W2" s="14"/>
+      <c r="X2" s="14"/>
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14"/>
+      <c r="AA2" s="14"/>
+      <c r="AB2" s="14"/>
+      <c r="AC2" s="14"/>
+      <c r="AD2" s="14"/>
+      <c r="AE2" s="14"/>
+      <c r="AF2" s="14"/>
+      <c r="AG2" s="14"/>
+      <c r="AH2" s="14"/>
+      <c r="AI2" s="14"/>
+      <c r="AJ2" s="14"/>
+      <c r="AK2" s="14"/>
+      <c r="AL2" s="14"/>
+      <c r="AM2" s="14"/>
+      <c r="AN2" s="14"/>
+      <c r="AO2" s="14"/>
+      <c r="AP2" s="14"/>
+      <c r="AQ2" s="14"/>
+      <c r="AR2" s="14"/>
+      <c r="AS2" s="14"/>
+      <c r="AT2" s="14"/>
+      <c r="AU2" s="14"/>
     </row>
     <row r="3" spans="1:47">
       <c r="E3" s="1"/>
@@ -3950,10 +4007,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="115.5" customHeight="1">
-      <c r="A1" s="10"/>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
+      <c r="A1" s="11"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
     </row>
     <row r="2" spans="1:4" ht="12.95" customHeight="1" thickBot="1">
       <c r="A2" s="4" t="s">
@@ -3979,7 +4036,7 @@
       <c r="C3" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -3993,8 +4050,8 @@
       <c r="C4" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>57</v>
+      <c r="D4" s="10" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="90.75" thickBot="1">
@@ -4007,7 +4064,7 @@
       <c r="C5" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4021,7 +4078,7 @@
       <c r="C6" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="10" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4035,7 +4092,7 @@
       <c r="C7" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4049,7 +4106,7 @@
       <c r="C8" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="13" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4063,7 +4120,7 @@
       <c r="C9" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="13" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4077,7 +4134,7 @@
       <c r="C10" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4091,7 +4148,7 @@
       <c r="C11" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4105,7 +4162,7 @@
       <c r="C12" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4119,7 +4176,7 @@
       <c r="C13" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4133,7 +4190,7 @@
       <c r="C14" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4147,7 +4204,7 @@
       <c r="C15" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4161,7 +4218,7 @@
       <c r="C16" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4175,7 +4232,7 @@
       <c r="C17" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="13" t="s">
         <v>92</v>
       </c>
     </row>
@@ -4189,7 +4246,7 @@
       <c r="C18" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4203,7 +4260,7 @@
       <c r="C19" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="10" t="s">
         <v>98</v>
       </c>
     </row>
@@ -4217,7 +4274,7 @@
       <c r="C20" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4231,7 +4288,7 @@
       <c r="C21" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4245,7 +4302,7 @@
       <c r="C22" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4259,7 +4316,7 @@
       <c r="C23" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4273,7 +4330,7 @@
       <c r="C24" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4287,7 +4344,7 @@
       <c r="C25" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="13" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4301,7 +4358,7 @@
       <c r="C26" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="D26" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4315,7 +4372,7 @@
       <c r="C27" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="D27" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4329,7 +4386,7 @@
       <c r="C28" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="D28" s="11" t="s">
+      <c r="D28" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4343,8 +4400,8 @@
       <c r="C29" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="D29" s="11" t="s">
-        <v>57</v>
+      <c r="D29" s="10" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60.75" thickBot="1">
@@ -4357,7 +4414,7 @@
       <c r="C30" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="13" t="s">
         <v>57</v>
       </c>
     </row>
@@ -4371,7 +4428,7 @@
       <c r="C31" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D31" s="12" t="s">
+      <c r="D31" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4385,7 +4442,7 @@
       <c r="C32" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4399,7 +4456,7 @@
       <c r="C33" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4413,7 +4470,7 @@
       <c r="C34" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D34" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4427,7 +4484,7 @@
       <c r="C35" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="D35" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4441,7 +4498,7 @@
       <c r="C36" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="D36" s="12" t="s">
+      <c r="D36" s="10" t="s">
         <v>136</v>
       </c>
     </row>
@@ -4455,7 +4512,7 @@
       <c r="C37" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="D37" s="12" t="s">
+      <c r="D37" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4469,7 +4526,7 @@
       <c r="C38" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="D38" s="12" t="s">
+      <c r="D38" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4483,7 +4540,7 @@
       <c r="C39" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="D39" s="12" t="s">
+      <c r="D39" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4497,7 +4554,7 @@
       <c r="C40" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="D40" s="10" t="s">
         <v>146</v>
       </c>
     </row>
@@ -4511,7 +4568,7 @@
       <c r="C41" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="D41" s="12" t="s">
+      <c r="D41" s="10" t="s">
         <v>146</v>
       </c>
     </row>
@@ -4525,7 +4582,7 @@
       <c r="C42" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="D42" s="12" t="s">
+      <c r="D42" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4539,7 +4596,7 @@
       <c r="C43" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4553,7 +4610,7 @@
       <c r="C44" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="D44" s="12" t="s">
+      <c r="D44" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4567,7 +4624,7 @@
       <c r="C45" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="D45" s="12" t="s">
+      <c r="D45" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4581,7 +4638,7 @@
       <c r="C46" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4595,7 +4652,7 @@
       <c r="C47" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="D47" s="12" t="s">
+      <c r="D47" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4609,7 +4666,7 @@
       <c r="C48" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="D48" s="12" t="s">
+      <c r="D48" s="10" t="s">
         <v>53</v>
       </c>
     </row>
@@ -4623,7 +4680,7 @@
       <c r="C49" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="D49" s="13" t="s">
+      <c r="D49" s="16" t="s">
         <v>57</v>
       </c>
     </row>

</xml_diff>